<commit_message>
Remove beans and rebalance existing foods
</commit_message>
<xml_diff>
--- a/Dieta.xlsx
+++ b/Dieta.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculadora" sheetId="1" r:id="R4f70359fb9d1439a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referências" sheetId="2" r:id="R8ab76e1291124fae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dieta" sheetId="3" r:id="R6b4925c517cc466b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rotina" sheetId="4" r:id="Rc7593e02655947b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculadora" sheetId="1" r:id="Rf3df1ed0e51f4cd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referências" sheetId="2" r:id="R0fd7fdec182f4b39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dieta" sheetId="3" r:id="R0968e2cb2cc448b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rotina" sheetId="4" r:id="R02598b9b04c04542"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -254,16 +254,6 @@
     <x:t xml:space="preserve">Almoço</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Arroz + feijão + frango + legumes + abacate</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Arroz cozido|350 g
-Feijão cozido|150 g
-Frango|120 g
-Legumes/salada|200 g
-Abacate|100 g</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">~75 g/dia</x:t>
   </x:si>
   <x:si>
@@ -342,23 +332,10 @@
     <x:t xml:space="preserve">Jantar / pós</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Arroz + feijão + carne + batata + legumes</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Arroz cozido|300 g
-Feijão|100 g
-Carne bovina magra|120 g
-Batata cozida/assada|100 g
-Legumes/salada|200 g</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">3. Almoço</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Arroz cozido</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">250 g</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">22h30</x:t>
@@ -372,12 +349,6 @@
   <x:si>
     <x:t xml:space="preserve">Leite|250 ml
 Manga|150 g</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Feijão cozido</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">150 g</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Terça</x:t>
@@ -393,19 +364,7 @@
 Banana|1 média</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Frango</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">~80 g</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">10h15</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Brócolis + couve-flor + alface</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">à vontade / ~200 g</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">11h20</x:t>
@@ -421,9 +380,6 @@
 Banana|1 média</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Abacate</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">12h00–13h00</x:t>
   </x:si>
   <x:si>
@@ -437,13 +393,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Almoço / pós</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Arroz cozido|350 g
-Feijão cozido|150 g
-Frango|120 g
-Legumes/salada|200 g
-Abacate|80 g</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Muçarela ou queijo prato</x:t>
@@ -472,26 +421,10 @@
     <x:t xml:space="preserve">20h15</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Arroz cozido|300 g
-Feijão|100 g
-Carne bovina magra|120 g
-Batata|100 g
-Legumes/salada|200 g</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">5. Jantar / pós-treino</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">200 g</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">22h15</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Feijão</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">100 g</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Quarta</x:t>
@@ -504,25 +437,6 @@
 Banana|1 média</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Carne bovina magra</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Batata cozida/assada</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Arroz + feijão + carne + legumes + abacate</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Arroz cozido|350 g
-Feijão|150 g
-Carne bovina magra|120 g
-Legumes/salada|200 g
-Abacate|100 g</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Brócolis/couve-flor/alface</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">6. Ceia</x:t>
   </x:si>
   <x:si>
@@ -532,27 +446,10 @@
     <x:t xml:space="preserve">~150 g</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Arroz + feijão + frango + batata + legumes</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Arroz cozido|300 g
-Feijão|100 g
-Frango|120 g
-Batata|100 g
-Legumes/salada|200 g</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Quinta — presencial</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Marmita</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Arroz cozido|350 g
-Feijão|150 g
-Frango|120 g
-Legumes|200 g
-Abacate|80 g</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Lanche no trabalho</x:t>
@@ -594,13 +491,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Sexta — presencial</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Arroz cozido|350 g
-Feijão|150 g
-Carne bovina magra|120 g
-Legumes|200 g
-Abacate|80 g</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">16h15</x:t>
@@ -635,13 +525,6 @@
 Whey|30 g</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Arroz cozido|350 g
-Feijão|150 g
-Frango|120 g
-Legumes/salada|200 g
-Abacate|100 g</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Pão + queijo + banana + uva</x:t>
   </x:si>
   <x:si>
@@ -676,32 +559,12 @@
     <x:t xml:space="preserve">12h30</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Arroz + feijão + carne + batata + legumes + abacate</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Arroz cozido|350 g
-Feijão|150 g
-Carne bovina magra|120 g
-Batata|100 g
-Legumes/salada|200 g
-Abacate|80 g</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Whey + mamão + pão</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Whey|30 g
 Mamão|200 g
 Pão|2 fatias</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Arroz + feijão + frango + legumes</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Arroz cozido|300 g
-Feijão|100 g
-Frango|120 g
-Legumes/salada|200 g</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">em casa</x:t>
@@ -2514,153 +2377,159 @@
       <x:c r="G4" s="27" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="H4" s="28" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="I4" s="68" t="s">
-        <x:v>79</x:v>
+      <x:c r="H4" s="28" t="str">
+        <x:v>Arroz + frango + legumes + abacate</x:v>
+      </x:c>
+      <x:c r="I4" s="68" t="str">
+        <x:v>Arroz cozido|410 g
+Frango|135 g
+Legumes/salada|300 g
+Abacate|100 g</x:v>
       </x:c>
       <x:c r="K4" s="2" t="s">
         <x:v>30</x:v>
       </x:c>
       <x:c r="L4" s="2" t="s">
-        <x:v>80</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="43.20000076293945">
       <x:c r="A5" s="94"/>
       <x:c r="B5" s="27" t="s">
-        <x:v>81</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="C5" s="28" t="s">
-        <x:v>82</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="E5" s="96"/>
       <x:c r="F5" s="58" t="s">
-        <x:v>83</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="G5" s="58" t="s">
         <x:v>72</x:v>
       </x:c>
       <x:c r="H5" s="59" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="I5" s="68" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="K5" s="2" t="s">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="I5" s="68" t="s">
+      <x:c r="L5" s="2" t="s">
         <x:v>85</x:v>
-      </x:c>
-      <x:c r="K5" s="2" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="L5" s="2" t="s">
-        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28.799999237060547">
       <x:c r="A6" s="93"/>
       <x:c r="B6" s="29" t="s">
-        <x:v>88</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="C6" s="30" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="E6" s="96"/>
       <x:c r="F6" s="27" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="G6" s="27" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="H6" s="28" t="s">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="G6" s="27" t="s">
+      <x:c r="I6" s="68" t="s">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="H6" s="28" t="s">
+      <x:c r="K6" s="2" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="I6" s="68" t="s">
+      <x:c r="L6" s="2" t="s">
         <x:v>93</x:v>
-      </x:c>
-      <x:c r="K6" s="2" t="s">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="L6" s="2" t="s">
-        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="92" t="s">
-        <x:v>96</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="B7" s="25" t="s">
-        <x:v>97</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="C7" s="26" t="s">
         <x:v>70</x:v>
       </x:c>
       <x:c r="E7" s="99"/>
       <x:c r="F7" s="75" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="G7" s="78" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="H7" s="76" t="s">
         <x:v>98</x:v>
-      </x:c>
-      <x:c r="G7" s="78" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="H7" s="76" t="s">
-        <x:v>100</x:v>
       </x:c>
       <x:c r="I7" s="77"/>
     </x:row>
     <x:row r="8" ht="72">
       <x:c r="A8" s="93"/>
       <x:c r="B8" s="29" t="s">
-        <x:v>101</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="C8" s="30" t="s">
-        <x:v>102</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="E8" s="95"/>
       <x:c r="F8" s="25" t="s">
-        <x:v>103</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="G8" s="25" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="H8" s="26" t="s">
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="I8" s="68" t="s">
-        <x:v>106</x:v>
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="H8" s="26" t="str">
+        <x:v>Arroz + carne + batata + legumes</x:v>
+      </x:c>
+      <x:c r="I8" s="68" t="str">
+        <x:v>Arroz cozido|335 g
+Carne bovina magra|127 g
+Batata cozida/assada|100 g
+Legumes/salada|300 g</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28.799999237060547">
       <x:c r="A9" s="92" t="s">
-        <x:v>107</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="B9" s="25" t="s">
-        <x:v>108</x:v>
-      </x:c>
-      <x:c r="C9" s="26" t="s">
-        <x:v>109</x:v>
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="C9" s="26" t="str">
+        <x:v>310 g</x:v>
       </x:c>
       <x:c r="E9" s="96"/>
       <x:c r="F9" s="58" t="s">
-        <x:v>110</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="G9" s="58" t="s">
-        <x:v>111</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="H9" s="59" t="s">
-        <x:v>112</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="I9" s="68" t="s">
-        <x:v>113</x:v>
+        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="72">
       <x:c r="A10" s="94"/>
-      <x:c r="B10" s="27" t="s">
-        <x:v>114</x:v>
-      </x:c>
-      <x:c r="C10" s="28" t="s">
-        <x:v>115</x:v>
+      <x:c r="B10" s="27" t="str">
+        <x:v>Frango</x:v>
+      </x:c>
+      <x:c r="C10" s="28" t="str">
+        <x:v>~95 g</x:v>
       </x:c>
       <x:c r="E10" s="96" t="s">
-        <x:v>116</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="F10" s="27" t="s">
         <x:v>63</x:v>
@@ -2669,23 +2538,23 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="H10" s="28" t="s">
-        <x:v>117</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="I10" s="68" t="s">
-        <x:v>118</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="28.799999237060547">
       <x:c r="A11" s="94"/>
-      <x:c r="B11" s="27" t="s">
-        <x:v>119</x:v>
-      </x:c>
-      <x:c r="C11" s="28" t="s">
-        <x:v>120</x:v>
+      <x:c r="B11" s="27" t="str">
+        <x:v>Brócolis + couve-flor + alface</x:v>
+      </x:c>
+      <x:c r="C11" s="28" t="str">
+        <x:v>~300 g</x:v>
       </x:c>
       <x:c r="E11" s="96"/>
       <x:c r="F11" s="58" t="s">
-        <x:v>121</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="G11" s="58" t="s">
         <x:v>72</x:v>
@@ -2702,49 +2571,45 @@
     </x:row>
     <x:row r="12" ht="28.799999237060547">
       <x:c r="A12" s="94"/>
-      <x:c r="B12" s="27" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="C12" s="28" t="s">
-        <x:v>123</x:v>
+      <x:c r="B12" s="27" t="str">
+        <x:v>Abacate</x:v>
+      </x:c>
+      <x:c r="C12" s="28" t="str">
+        <x:v>~80 g</x:v>
       </x:c>
       <x:c r="E12" s="96"/>
       <x:c r="F12" s="58" t="s">
-        <x:v>124</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="G12" s="58" t="s">
-        <x:v>125</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="H12" s="59" t="s">
-        <x:v>126</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="I12" s="68" t="s">
-        <x:v>127</x:v>
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="93"/>
-      <x:c r="B13" s="29" t="s">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="C13" s="30" t="s">
-        <x:v>120</x:v>
-      </x:c>
+      <x:c r="B13" s="29" t="str"/>
+      <x:c r="C13" s="30" t="str"/>
       <x:c r="E13" s="97"/>
       <x:c r="F13" s="79" t="s">
-        <x:v>129</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="G13" s="81" t="s">
-        <x:v>130</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="H13" s="80" t="s">
-        <x:v>100</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="I13" s="77"/>
     </x:row>
     <x:row r="14" ht="72">
       <x:c r="A14" s="92" t="s">
-        <x:v>131</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="B14" s="25" t="s">
         <x:v>60</x:v>
@@ -2754,116 +2619,122 @@
       </x:c>
       <x:c r="E14" s="98"/>
       <x:c r="F14" s="60" t="s">
-        <x:v>132</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="G14" s="60" t="s">
-        <x:v>133</x:v>
-      </x:c>
-      <x:c r="H14" s="61" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="I14" s="68" t="s">
-        <x:v>134</x:v>
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="H14" s="61" t="str">
+        <x:v>Arroz + frango + legumes + abacate</x:v>
+      </x:c>
+      <x:c r="I14" s="68" t="str">
+        <x:v>Arroz cozido|410 g
+Frango|135 g
+Legumes/salada|300 g
+Abacate|80 g</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="43.20000076293945">
       <x:c r="A15" s="94"/>
       <x:c r="B15" s="27" t="s">
-        <x:v>135</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="C15" s="28" t="s">
         <x:v>70</x:v>
       </x:c>
       <x:c r="E15" s="95"/>
       <x:c r="F15" s="25" t="s">
-        <x:v>83</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="G15" s="25" t="s">
-        <x:v>136</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="H15" s="26" t="s">
-        <x:v>84</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="I15" s="68" t="s">
-        <x:v>137</x:v>
+        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="94"/>
       <x:c r="B16" s="27" t="s">
-        <x:v>88</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="C16" s="28" t="s">
-        <x:v>89</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="E16" s="97"/>
       <x:c r="F16" s="79" t="s">
-        <x:v>138</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="G16" s="81" t="s">
-        <x:v>139</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="H16" s="80" t="s">
-        <x:v>100</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="I16" s="77"/>
     </x:row>
     <x:row r="17" ht="72">
       <x:c r="A17" s="93"/>
       <x:c r="B17" s="29" t="s">
-        <x:v>140</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="C17" s="30" t="s">
-        <x:v>141</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E17" s="96"/>
       <x:c r="F17" s="27" t="s">
-        <x:v>142</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="G17" s="27" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="H17" s="28" t="s">
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="I17" s="68" t="s">
-        <x:v>143</x:v>
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="H17" s="28" t="str">
+        <x:v>Arroz + carne + batata + legumes</x:v>
+      </x:c>
+      <x:c r="I17" s="68" t="str">
+        <x:v>Arroz cozido|335 g
+Carne bovina magra|127 g
+Batata|100 g
+Legumes/salada|300 g</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="28.799999237060547">
       <x:c r="A18" s="92" t="s">
-        <x:v>144</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="B18" s="25" t="s">
-        <x:v>108</x:v>
-      </x:c>
-      <x:c r="C18" s="26" t="s">
-        <x:v>145</x:v>
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="C18" s="26" t="str">
+        <x:v>235 g</x:v>
       </x:c>
       <x:c r="E18" s="96"/>
       <x:c r="F18" s="58" t="s">
-        <x:v>146</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="G18" s="58" t="s">
-        <x:v>111</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="H18" s="59" t="s">
-        <x:v>112</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="I18" s="68" t="s">
-        <x:v>113</x:v>
+        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="72">
       <x:c r="A19" s="94"/>
-      <x:c r="B19" s="27" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="C19" s="28" t="s">
-        <x:v>148</x:v>
+      <x:c r="B19" s="27" t="str">
+        <x:v>Carne bovina magra</x:v>
+      </x:c>
+      <x:c r="C19" s="28" t="str">
+        <x:v>~107 g</x:v>
       </x:c>
       <x:c r="E19" s="96" t="s">
-        <x:v>149</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="F19" s="27" t="s">
         <x:v>63</x:v>
@@ -2875,16 +2746,16 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="I19" s="68" t="s">
-        <x:v>150</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="28.799999237060547">
       <x:c r="A20" s="94"/>
-      <x:c r="B20" s="27" t="s">
-        <x:v>151</x:v>
-      </x:c>
-      <x:c r="C20" s="28" t="s">
-        <x:v>141</x:v>
+      <x:c r="B20" s="27" t="str">
+        <x:v>Batata cozida/assada</x:v>
+      </x:c>
+      <x:c r="C20" s="28" t="str">
+        <x:v>~100 g</x:v>
       </x:c>
       <x:c r="E20" s="98"/>
       <x:c r="F20" s="60" t="s">
@@ -2905,11 +2776,11 @@
     </x:row>
     <x:row r="21" ht="72">
       <x:c r="A21" s="94"/>
-      <x:c r="B21" s="27" t="s">
-        <x:v>152</x:v>
-      </x:c>
-      <x:c r="C21" s="28" t="s">
-        <x:v>141</x:v>
+      <x:c r="B21" s="27" t="str">
+        <x:v>Brócolis/couve-flor/alface</x:v>
+      </x:c>
+      <x:c r="C21" s="28" t="str">
+        <x:v>~300 g</x:v>
       </x:c>
       <x:c r="E21" s="95"/>
       <x:c r="F21" s="25" t="s">
@@ -2918,38 +2789,37 @@
       <x:c r="G21" s="25" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="H21" s="26" t="s">
-        <x:v>153</x:v>
-      </x:c>
-      <x:c r="I21" s="68" t="s">
-        <x:v>154</x:v>
+      <x:c r="H21" s="26" t="str">
+        <x:v>Arroz + carne + legumes + abacate</x:v>
+      </x:c>
+      <x:c r="I21" s="68" t="str">
+        <x:v>Arroz cozido|405 g
+Carne bovina magra|132 g
+Legumes/salada|300 g
+Abacate|100 g</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="43.20000076293945">
       <x:c r="A22" s="93"/>
-      <x:c r="B22" s="29" t="s">
-        <x:v>155</x:v>
-      </x:c>
-      <x:c r="C22" s="30" t="s">
-        <x:v>102</x:v>
-      </x:c>
+      <x:c r="B22" s="29" t="str"/>
+      <x:c r="C22" s="30" t="str"/>
       <x:c r="E22" s="96"/>
       <x:c r="F22" s="27" t="s">
-        <x:v>83</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="G22" s="27" t="s">
         <x:v>72</x:v>
       </x:c>
       <x:c r="H22" s="28" t="s">
-        <x:v>84</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="I22" s="68" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="28.799999237060547">
       <x:c r="A23" s="92" t="s">
-        <x:v>156</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="B23" s="25" t="s">
         <x:v>74</x:v>
@@ -2959,71 +2829,74 @@
       </x:c>
       <x:c r="E23" s="96"/>
       <x:c r="F23" s="27" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="G23" s="27" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="H23" s="28" t="s">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="G23" s="27" t="s">
+      <x:c r="I23" s="68" t="s">
         <x:v>91</x:v>
-      </x:c>
-      <x:c r="H23" s="28" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="I23" s="68" t="s">
-        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="93"/>
       <x:c r="B24" s="29" t="s">
-        <x:v>157</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C24" s="30" t="s">
-        <x:v>158</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="E24" s="97"/>
       <x:c r="F24" s="79" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="G24" s="81" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="H24" s="80" t="s">
         <x:v>98</x:v>
-      </x:c>
-      <x:c r="G24" s="81" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="H24" s="80" t="s">
-        <x:v>100</x:v>
       </x:c>
       <x:c r="I24" s="77"/>
     </x:row>
     <x:row r="25" ht="72">
       <x:c r="E25" s="96"/>
       <x:c r="F25" s="58" t="s">
-        <x:v>103</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="G25" s="58" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="H25" s="59" t="s">
-        <x:v>159</x:v>
-      </x:c>
-      <x:c r="I25" s="68" t="s">
-        <x:v>160</x:v>
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="H25" s="59" t="str">
+        <x:v>Arroz + frango + batata + legumes</x:v>
+      </x:c>
+      <x:c r="I25" s="68" t="str">
+        <x:v>Arroz cozido|335 g
+Frango|128 g
+Batata|100 g
+Legumes/salada|300 g</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="28.799999237060547">
       <x:c r="E26" s="96"/>
       <x:c r="F26" s="27" t="s">
-        <x:v>110</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="G26" s="27" t="s">
-        <x:v>111</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="H26" s="28" t="s">
-        <x:v>112</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="I26" s="68" t="s">
-        <x:v>113</x:v>
+        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="72">
       <x:c r="E27" s="98" t="s">
-        <x:v>161</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="F27" s="60" t="s">
         <x:v>63</x:v>
@@ -3035,7 +2908,7 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="I27" s="68" t="s">
-        <x:v>150</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="28.799999237060547">
@@ -3062,78 +2935,84 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="G29" s="27" t="s">
-        <x:v>162</x:v>
-      </x:c>
-      <x:c r="H29" s="28" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="I29" s="68" t="s">
-        <x:v>163</x:v>
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="H29" s="28" t="str">
+        <x:v>Arroz + frango + legumes + abacate</x:v>
+      </x:c>
+      <x:c r="I29" s="68" t="str">
+        <x:v>Arroz cozido|410 g
+Frango|135 g
+Legumes|300 g
+Abacate|80 g</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="43.20000076293945">
       <x:c r="E30" s="96"/>
       <x:c r="F30" s="27" t="s">
-        <x:v>83</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="G30" s="27" t="s">
-        <x:v>164</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="H30" s="28" t="s">
-        <x:v>165</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="I30" s="68" t="s">
-        <x:v>166</x:v>
+        <x:v>141</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="43.20000076293945">
       <x:c r="E31" s="96"/>
       <x:c r="F31" s="27" t="s">
-        <x:v>167</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="G31" s="27" t="s">
-        <x:v>168</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="H31" s="28" t="s">
-        <x:v>169</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="I31" s="68" t="s">
-        <x:v>170</x:v>
+        <x:v>145</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="72">
       <x:c r="E32" s="96"/>
       <x:c r="F32" s="58" t="s">
-        <x:v>171</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="G32" s="58" t="s">
-        <x:v>172</x:v>
-      </x:c>
-      <x:c r="H32" s="59" t="s">
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="I32" s="68" t="s">
-        <x:v>143</x:v>
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="H32" s="59" t="str">
+        <x:v>Arroz + carne + batata + legumes</x:v>
+      </x:c>
+      <x:c r="I32" s="68" t="str">
+        <x:v>Arroz cozido|335 g
+Carne bovina magra|127 g
+Batata|100 g
+Legumes/salada|300 g</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="28.799999237060547">
       <x:c r="E33" s="96"/>
       <x:c r="F33" s="27" t="s">
-        <x:v>110</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="G33" s="27" t="s">
-        <x:v>111</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="H33" s="28" t="s">
-        <x:v>173</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="I33" s="68" t="s">
-        <x:v>174</x:v>
+        <x:v>149</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="72">
       <x:c r="E34" s="98" t="s">
-        <x:v>175</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="F34" s="60" t="s">
         <x:v>63</x:v>
@@ -3145,7 +3024,7 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="I34" s="68" t="s">
-        <x:v>150</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="28.799999237060547">
@@ -3172,131 +3051,137 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="G36" s="27" t="s">
-        <x:v>162</x:v>
-      </x:c>
-      <x:c r="H36" s="28" t="s">
-        <x:v>153</x:v>
-      </x:c>
-      <x:c r="I36" s="68" t="s">
-        <x:v>176</x:v>
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="H36" s="28" t="str">
+        <x:v>Arroz + carne + legumes + abacate</x:v>
+      </x:c>
+      <x:c r="I36" s="68" t="str">
+        <x:v>Arroz cozido|405 g
+Carne bovina magra|132 g
+Legumes|300 g
+Abacate|80 g</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="43.20000076293945">
       <x:c r="E37" s="96"/>
       <x:c r="F37" s="58" t="s">
-        <x:v>177</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="G37" s="58" t="s">
         <x:v>72</x:v>
       </x:c>
       <x:c r="H37" s="59" t="s">
-        <x:v>84</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="I37" s="68" t="s">
-        <x:v>85</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="28.799999237060547">
       <x:c r="E38" s="96"/>
       <x:c r="F38" s="27" t="s">
-        <x:v>178</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="G38" s="27" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="H38" s="28" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="I38" s="68" t="s">
         <x:v>91</x:v>
-      </x:c>
-      <x:c r="H38" s="28" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="I38" s="68" t="s">
-        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="E39" s="97"/>
       <x:c r="F39" s="79" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="G39" s="81" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="H39" s="80" t="s">
         <x:v>98</x:v>
-      </x:c>
-      <x:c r="G39" s="81" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="H39" s="80" t="s">
-        <x:v>100</x:v>
       </x:c>
       <x:c r="I39" s="77"/>
     </x:row>
     <x:row r="40" ht="72">
       <x:c r="E40" s="98"/>
       <x:c r="F40" s="29" t="s">
-        <x:v>103</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="G40" s="29" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="H40" s="30" t="s">
-        <x:v>159</x:v>
-      </x:c>
-      <x:c r="I40" s="68" t="s">
-        <x:v>160</x:v>
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="H40" s="30" t="str">
+        <x:v>Arroz + frango + batata + legumes</x:v>
+      </x:c>
+      <x:c r="I40" s="68" t="str">
+        <x:v>Arroz cozido|335 g
+Frango|128 g
+Batata|100 g
+Legumes/salada|300 g</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="28.799999237060547">
       <x:c r="E41" s="95"/>
       <x:c r="F41" s="25" t="s">
-        <x:v>110</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="G41" s="25" t="s">
-        <x:v>111</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="H41" s="26" t="s">
-        <x:v>112</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="I41" s="68" t="s">
-        <x:v>113</x:v>
+        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="28.799999237060547">
       <x:c r="E42" s="96" t="s">
-        <x:v>179</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="F42" s="58" t="s">
-        <x:v>180</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="G42" s="58" t="s">
-        <x:v>125</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="H42" s="59" t="s">
-        <x:v>92</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="I42" s="68" t="s">
-        <x:v>93</x:v>
+        <x:v>91</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="E43" s="97"/>
       <x:c r="F43" s="79" t="s">
-        <x:v>181</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="G43" s="81" t="s">
-        <x:v>130</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="H43" s="80" t="s">
-        <x:v>100</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="I43" s="77"/>
     </x:row>
     <x:row r="44" ht="86.4000015258789">
       <x:c r="E44" s="96"/>
       <x:c r="F44" s="58" t="s">
-        <x:v>182</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="G44" s="58" t="s">
-        <x:v>183</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="H44" s="59" t="s">
-        <x:v>184</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="I44" s="68" t="s">
-        <x:v>185</x:v>
+        <x:v>159</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="72">
@@ -3307,64 +3192,70 @@
       <x:c r="G45" s="27" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="H45" s="28" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="I45" s="68" t="s">
-        <x:v>186</x:v>
+      <x:c r="H45" s="28" t="str">
+        <x:v>Arroz + frango + legumes + abacate</x:v>
+      </x:c>
+      <x:c r="I45" s="68" t="str">
+        <x:v>Arroz cozido|410 g
+Frango|135 g
+Legumes/salada|300 g
+Abacate|100 g</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="57.599998474121094">
       <x:c r="E46" s="98"/>
       <x:c r="F46" s="29" t="s">
-        <x:v>83</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="G46" s="29" t="s">
         <x:v>72</x:v>
       </x:c>
       <x:c r="H46" s="30" t="s">
-        <x:v>187</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="I46" s="68" t="s">
-        <x:v>188</x:v>
+        <x:v>161</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="72">
       <x:c r="E47" s="71"/>
       <x:c r="F47" s="73" t="s">
-        <x:v>189</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="G47" s="2" t="s">
-        <x:v>172</x:v>
-      </x:c>
-      <x:c r="H47" s="2" t="s">
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="I47" s="68" t="s">
-        <x:v>143</x:v>
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="H47" s="2" t="str">
+        <x:v>Arroz + carne + batata + legumes</x:v>
+      </x:c>
+      <x:c r="I47" s="68" t="str">
+        <x:v>Arroz cozido|335 g
+Carne bovina magra|127 g
+Batata|100 g
+Legumes/salada|300 g</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="28.799999237060547">
       <x:c r="E48" s="71"/>
       <x:c r="F48" s="73" t="s">
-        <x:v>110</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="G48" s="2" t="s">
-        <x:v>111</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="H48" s="2" t="s">
-        <x:v>112</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="I48" s="68" t="s">
-        <x:v>113</x:v>
+        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="72">
       <x:c r="E49" s="71" t="s">
-        <x:v>190</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="F49" s="73" t="s">
-        <x:v>191</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="G49" s="2" t="s">
         <x:v>64</x:v>
@@ -3373,95 +3264,101 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="I49" s="68" t="s">
-        <x:v>150</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="28.799999237060547">
       <x:c r="E50" s="71"/>
       <x:c r="F50" s="73" t="s">
-        <x:v>192</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="G50" s="2" t="s">
-        <x:v>125</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="H50" s="2" t="s">
-        <x:v>193</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="I50" s="68" t="s">
-        <x:v>194</x:v>
+        <x:v>167</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="E51" s="82"/>
       <x:c r="F51" s="83" t="s">
-        <x:v>195</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="G51" s="85" t="s">
-        <x:v>130</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="H51" s="84" t="s">
-        <x:v>100</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="I51" s="77"/>
     </x:row>
     <x:row r="52" ht="86.4000015258789">
       <x:c r="E52" s="71"/>
       <x:c r="F52" s="73" t="s">
-        <x:v>196</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="G52" s="2" t="s">
-        <x:v>133</x:v>
-      </x:c>
-      <x:c r="H52" s="2" t="s">
-        <x:v>197</x:v>
-      </x:c>
-      <x:c r="I52" s="68" t="s">
-        <x:v>198</x:v>
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="H52" s="2" t="str">
+        <x:v>Arroz + carne + batata + legumes + abacate</x:v>
+      </x:c>
+      <x:c r="I52" s="68" t="str">
+        <x:v>Arroz cozido|405 g
+Carne bovina magra|132 g
+Batata|100 g
+Legumes/salada|300 g
+Abacate|80 g</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="43.20000076293945">
       <x:c r="E53" s="71"/>
       <x:c r="F53" s="73" t="s">
-        <x:v>83</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="G53" s="2" t="s">
         <x:v>72</x:v>
       </x:c>
       <x:c r="H53" s="2" t="s">
-        <x:v>199</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="I53" s="68" t="s">
-        <x:v>200</x:v>
+        <x:v>171</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="57.599998474121094">
       <x:c r="E54" s="71"/>
       <x:c r="F54" s="73" t="s">
-        <x:v>189</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="G54" s="2" t="s">
-        <x:v>172</x:v>
-      </x:c>
-      <x:c r="H54" s="2" t="s">
-        <x:v>201</x:v>
-      </x:c>
-      <x:c r="I54" s="68" t="s">
-        <x:v>202</x:v>
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="H54" s="2" t="str">
+        <x:v>Arroz + frango + legumes</x:v>
+      </x:c>
+      <x:c r="I54" s="68" t="str">
+        <x:v>Arroz cozido|335 g
+Frango|128 g
+Legumes/salada|300 g</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="28.799999237060547">
       <x:c r="E55" s="72"/>
       <x:c r="F55" s="74" t="s">
-        <x:v>146</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="G55" s="69" t="s">
-        <x:v>111</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="H55" s="69" t="s">
-        <x:v>112</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="I55" s="70" t="s">
-        <x:v>113</x:v>
+        <x:v>108</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3501,33 +3398,33 @@
     <x:row r="2">
       <x:c r="A2" s="34"/>
       <x:c r="B2" s="35" t="s">
-        <x:v>203</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="C2" s="35" t="s">
-        <x:v>203</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="D2" s="36" t="s">
-        <x:v>203</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="H2" s="50" t="s">
-        <x:v>204</x:v>
+        <x:v>173</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="37" t="s">
-        <x:v>205</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="B3" s="39" t="s">
-        <x:v>206</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="C3" s="39" t="s">
-        <x:v>207</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="D3" s="38" t="s">
-        <x:v>208</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="H3" s="49" t="s">
-        <x:v>209</x:v>
+        <x:v>178</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -3535,16 +3432,16 @@
         <x:v>0.22916666666666666</x:v>
       </x:c>
       <x:c r="B4" s="41" t="s">
-        <x:v>210</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="C4" s="41" t="s">
-        <x:v>210</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="D4" s="42" t="s">
-        <x:v>210</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="H4" s="52" t="s">
-        <x:v>211</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -3552,16 +3449,16 @@
         <x:v>0.27083333333333331</x:v>
       </x:c>
       <x:c r="B5" s="41" t="s">
-        <x:v>212</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="C5" s="41" t="s">
-        <x:v>212</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="D5" s="42" t="s">
-        <x:v>212</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="H5" s="53" t="s">
-        <x:v>213</x:v>
+        <x:v>182</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -3569,13 +3466,13 @@
         <x:v>0.33333333333333331</x:v>
       </x:c>
       <x:c r="B6" s="41" t="s">
-        <x:v>214</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="C6" s="41" t="s">
-        <x:v>214</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="D6" s="42" t="s">
-        <x:v>214</x:v>
+        <x:v>183</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -3583,13 +3480,13 @@
         <x:v>0.375</x:v>
       </x:c>
       <x:c r="B7" s="51" t="s">
-        <x:v>215</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="C7" s="41" t="s">
-        <x:v>215</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="D7" s="42" t="s">
-        <x:v>215</x:v>
+        <x:v>184</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -3597,13 +3494,13 @@
         <x:v>0.54166666666666663</x:v>
       </x:c>
       <x:c r="B8" s="51" t="s">
-        <x:v>216</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="C8" s="51" t="s">
-        <x:v>217</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="D8" s="54" t="s">
-        <x:v>216</x:v>
+        <x:v>185</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -3611,13 +3508,13 @@
         <x:v>0.58333333333333337</x:v>
       </x:c>
       <x:c r="B9" s="51" t="s">
-        <x:v>215</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="C9" s="51" t="s">
-        <x:v>215</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="D9" s="42" t="s">
-        <x:v>215</x:v>
+        <x:v>184</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -3625,13 +3522,13 @@
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="B10" s="51" t="s">
-        <x:v>218</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="C10" s="102" t="s">
-        <x:v>211</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="D10" s="42" t="s">
-        <x:v>218</x:v>
+        <x:v>187</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -3639,11 +3536,11 @@
         <x:v>0.79166666666666663</x:v>
       </x:c>
       <x:c r="B11" s="104" t="s">
-        <x:v>209</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="C11" s="102"/>
       <x:c r="D11" s="103" t="s">
-        <x:v>209</x:v>
+        <x:v>178</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -3652,7 +3549,7 @@
       </x:c>
       <x:c r="B12" s="104"/>
       <x:c r="C12" s="51" t="s">
-        <x:v>219</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="D12" s="103"/>
     </x:row>
@@ -3661,62 +3558,62 @@
         <x:v>0.91666666666666663</x:v>
       </x:c>
       <x:c r="B13" s="24" t="s">
-        <x:v>220</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="C13" s="48" t="s">
-        <x:v>220</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="D13" s="46" t="s">
-        <x:v>220</x:v>
+        <x:v>189</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="40" t="s">
-        <x:v>221</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="B14" s="57" t="s">
-        <x:v>222</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="C14" s="56" t="s">
-        <x:v>222</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="D14" s="43" t="s">
-        <x:v>222</x:v>
+        <x:v>191</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15">
       <x:c r="A15" s="47" t="s">
-        <x:v>221</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="B15" s="55" t="s">
-        <x:v>223</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="C15" s="48" t="s">
-        <x:v>223</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="D15" s="45" t="s">
-        <x:v>223</x:v>
+        <x:v>192</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15"/>
     <x:row r="17" ht="15">
       <x:c r="A17" s="34"/>
       <x:c r="B17" s="35" t="s">
-        <x:v>224</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="C17" s="36" t="s">
-        <x:v>224</x:v>
+        <x:v>193</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15">
       <x:c r="A18" s="37" t="s">
-        <x:v>205</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="B18" s="39" t="s">
-        <x:v>225</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="C18" s="38" t="s">
-        <x:v>226</x:v>
+        <x:v>195</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -3724,10 +3621,10 @@
         <x:v>0.22916666666666666</x:v>
       </x:c>
       <x:c r="B19" s="51" t="s">
-        <x:v>213</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="C19" s="42" t="s">
-        <x:v>210</x:v>
+        <x:v>179</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -3735,10 +3632,10 @@
         <x:v>0.33333333333333331</x:v>
       </x:c>
       <x:c r="B20" s="41" t="s">
-        <x:v>215</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="C20" s="42" t="s">
-        <x:v>215</x:v>
+        <x:v>184</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -3746,10 +3643,10 @@
         <x:v>0.54166666666666663</x:v>
       </x:c>
       <x:c r="B21" s="51" t="s">
-        <x:v>227</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="C21" s="54" t="s">
-        <x:v>228</x:v>
+        <x:v>197</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -3757,10 +3654,10 @@
         <x:v>0.58333333333333337</x:v>
       </x:c>
       <x:c r="B22" s="41" t="s">
-        <x:v>215</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="C22" s="42" t="s">
-        <x:v>215</x:v>
+        <x:v>184</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -3768,10 +3665,10 @@
         <x:v>0.79166666666666663</x:v>
       </x:c>
       <x:c r="B23" s="24" t="s">
-        <x:v>229</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="C23" s="103" t="s">
-        <x:v>209</x:v>
+        <x:v>178</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -3779,7 +3676,7 @@
         <x:v>0.83333333333333337</x:v>
       </x:c>
       <x:c r="B24" s="24" t="s">
-        <x:v>216</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="C24" s="103"/>
     </x:row>
@@ -3788,30 +3685,30 @@
         <x:v>0.91666666666666663</x:v>
       </x:c>
       <x:c r="B25" s="24" t="s">
-        <x:v>220</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="C25" s="46" t="s">
-        <x:v>220</x:v>
+        <x:v>189</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="100" t="s">
-        <x:v>221</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="B26" s="56" t="s">
-        <x:v>222</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="C26" s="43" t="s">
-        <x:v>222</x:v>
+        <x:v>191</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="101"/>
       <x:c r="B27" s="48" t="s">
-        <x:v>223</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="C27" s="45" t="s">
-        <x:v>223</x:v>
+        <x:v>192</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>